<commit_message>
Uploading the shapefiles for the survey stations and deleting and replacing the order of the output folder to contain "abundance" and "P-A" for the different dataset outputs
</commit_message>
<xml_diff>
--- a/data/grab_data/grabsites.xlsx
+++ b/data/grab_data/grabsites.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sarahstevenson/Desktop/diss/SouthArran/data/grab_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A83152-1051-D34F-A265-20C6935AF21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3765D7-2B3F-9145-B7A3-87CCD27A6527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4400" yWindow="520" windowWidth="24180" windowHeight="15720" xr2:uid="{D8AFAFA6-CD89-D240-A7BB-2EF4CF0946D6}"/>
   </bookViews>
@@ -977,7 +977,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -985,6 +985,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5943,28 +5947,28 @@
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A192" s="2" t="s">
+      <c r="A192" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B192">
-        <v>2022</v>
-      </c>
-      <c r="C192">
+      <c r="B192" s="4">
+        <v>2022</v>
+      </c>
+      <c r="C192" s="4">
         <v>55.578164999999998</v>
       </c>
-      <c r="D192">
+      <c r="D192" s="4">
         <v>-5.0751217000000004</v>
       </c>
-      <c r="E192" s="3" t="s">
+      <c r="E192" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="F192" t="s">
+      <c r="F192" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="G192">
+      <c r="G192" s="4">
         <v>4.9221149999999998</v>
       </c>
-      <c r="H192">
+      <c r="H192" s="4">
         <v>4.7988479999999996</v>
       </c>
     </row>
@@ -6035,21 +6039,24 @@
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A196" s="2" t="s">
+      <c r="A196" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B196">
-        <v>2022</v>
-      </c>
-      <c r="C196">
+      <c r="B196" s="4">
+        <v>2022</v>
+      </c>
+      <c r="C196" s="4">
         <v>55.5696133</v>
       </c>
-      <c r="D196">
+      <c r="D196" s="4">
         <v>-5.0652566999999999</v>
       </c>
-      <c r="E196" s="3" t="s">
+      <c r="E196" s="6" t="s">
         <v>275</v>
       </c>
+      <c r="F196" s="4"/>
+      <c r="G196" s="4"/>
+      <c r="H196" s="4"/>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="2" t="s">

</xml_diff>

<commit_message>
updated files - filled in 2022 data for T survey sites - re-run BTA empty matrix for PA and abundance counts - Filled in matrix for abundance
</commit_message>
<xml_diff>
--- a/data/grab_data/grabsites.xlsx
+++ b/data/grab_data/grabsites.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sarahstevenson/Desktop/diss/SouthArran/data/grab_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9FB5D1F-F4EF-484C-A511-A1804E609ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851C8D70-6B51-8A42-8C3D-7939EEF85C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="520" windowWidth="24180" windowHeight="15720" xr2:uid="{D8AFAFA6-CD89-D240-A7BB-2EF4CF0946D6}"/>
+    <workbookView xWindow="4620" yWindow="500" windowWidth="24180" windowHeight="15720" xr2:uid="{D8AFAFA6-CD89-D240-A7BB-2EF4CF0946D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="241">
   <si>
     <t>G01</t>
   </si>
@@ -697,18 +697,6 @@
     <t>D3_G09-1</t>
   </si>
   <si>
-    <t>D1_02-1</t>
-  </si>
-  <si>
-    <t>D1_02-2</t>
-  </si>
-  <si>
-    <t>D1_03-1</t>
-  </si>
-  <si>
-    <t>D1_03-2</t>
-  </si>
-  <si>
     <t>D6G04</t>
   </si>
   <si>
@@ -754,27 +742,9 @@
     <t>T1G8 </t>
   </si>
   <si>
-    <t>Fine Sand</t>
-  </si>
-  <si>
-    <t>Medium Sand</t>
-  </si>
-  <si>
     <t>Coarse Sand</t>
   </si>
   <si>
-    <t>Very Coarse Sand</t>
-  </si>
-  <si>
-    <t>Very Coarse Silt</t>
-  </si>
-  <si>
-    <t>Coarse Silt</t>
-  </si>
-  <si>
-    <t>Very Fine Sand</t>
-  </si>
-  <si>
     <t>Medium silt</t>
   </si>
   <si>
@@ -782,6 +752,12 @@
   </si>
   <si>
     <t>D3_G09-2</t>
+  </si>
+  <si>
+    <t>D1_02</t>
+  </si>
+  <si>
+    <t>D1_03</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF0B1962-1941-1A4C-8A4B-C9F3C252480E}">
-  <dimension ref="A1:H238"/>
+  <dimension ref="A1:H236"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15.33203125" style="1" customWidth="1"/>
@@ -1207,7 +1183,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="F1" t="s">
         <v>10</v>
@@ -1288,7 +1264,7 @@
         <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G4">
         <v>-0.84</v>
@@ -1314,7 +1290,7 @@
         <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G5">
         <v>4.3600000000000003</v>
@@ -1340,7 +1316,7 @@
         <v>119</v>
       </c>
       <c r="F6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G6">
         <v>5.04</v>
@@ -1418,7 +1394,7 @@
         <v>77.400000000000006</v>
       </c>
       <c r="F9" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G9">
         <v>5.76</v>
@@ -1444,7 +1420,7 @@
         <v>22.5</v>
       </c>
       <c r="F10" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G10">
         <v>-0.17</v>
@@ -1470,7 +1446,7 @@
         <v>22.5</v>
       </c>
       <c r="F11" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G11">
         <v>-0.85</v>
@@ -1496,7 +1472,7 @@
         <v>22.5</v>
       </c>
       <c r="F12" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G12">
         <v>-0.24</v>
@@ -1626,7 +1602,7 @@
         <v>14.6</v>
       </c>
       <c r="F17" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="G17">
         <v>-1.6</v>
@@ -1652,7 +1628,7 @@
         <v>18.600000000000001</v>
       </c>
       <c r="F18" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="G18">
         <v>-2.02</v>
@@ -1880,7 +1856,7 @@
         <v>18.2</v>
       </c>
       <c r="F27" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="G27">
         <v>-5.71</v>
@@ -1906,7 +1882,7 @@
         <v>24.2</v>
       </c>
       <c r="F28" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G28">
         <v>-0.02</v>
@@ -2036,7 +2012,7 @@
         <v>12.3</v>
       </c>
       <c r="F33" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G33">
         <v>1.31</v>
@@ -2062,7 +2038,7 @@
         <v>17</v>
       </c>
       <c r="F34" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G34">
         <v>1.1499999999999999</v>
@@ -2114,7 +2090,7 @@
         <v>84.3</v>
       </c>
       <c r="F36" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G36">
         <v>4.8899999999999997</v>
@@ -2140,7 +2116,7 @@
         <v>102.5</v>
       </c>
       <c r="F37" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G37">
         <v>5.36</v>
@@ -2166,7 +2142,7 @@
         <v>13.4</v>
       </c>
       <c r="F38" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G38">
         <v>0.15</v>
@@ -2192,7 +2168,7 @@
         <v>13.4</v>
       </c>
       <c r="F39" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G39">
         <v>-0.5</v>
@@ -2218,7 +2194,7 @@
         <v>13.4</v>
       </c>
       <c r="F40" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G40">
         <v>-0.57999999999999996</v>
@@ -2270,7 +2246,7 @@
         <v>74.3</v>
       </c>
       <c r="F42" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G42">
         <v>3.99</v>
@@ -2296,7 +2272,7 @@
         <v>103.7</v>
       </c>
       <c r="F43" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G43">
         <v>6.01</v>
@@ -2322,7 +2298,7 @@
         <v>86.3</v>
       </c>
       <c r="F44" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G44">
         <v>5.73</v>
@@ -2582,7 +2558,7 @@
         <v>9.3000000000000007</v>
       </c>
       <c r="F54" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G54">
         <v>-0.72</v>
@@ -2608,7 +2584,7 @@
         <v>10.4</v>
       </c>
       <c r="F55" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G55">
         <v>0.8</v>
@@ -2764,7 +2740,7 @@
         <v>16</v>
       </c>
       <c r="F61" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G61">
         <v>-0.99</v>
@@ -2816,7 +2792,7 @@
         <v>4</v>
       </c>
       <c r="F63" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G63">
         <v>-1.73</v>
@@ -2868,7 +2844,7 @@
         <v>5.3</v>
       </c>
       <c r="F65" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G65">
         <v>0.11</v>
@@ -2920,7 +2896,7 @@
         <v>10.4</v>
       </c>
       <c r="F67" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G67">
         <v>-0.17</v>
@@ -2998,7 +2974,7 @@
         <v>3.9</v>
       </c>
       <c r="F70" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="G70">
         <v>-2.1800000000000002</v>
@@ -3061,7 +3037,7 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B73" s="1">
         <v>42200</v>
@@ -3087,7 +3063,7 @@
     </row>
     <row r="74" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B74" s="1">
         <v>42200</v>
@@ -3113,7 +3089,7 @@
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B75" s="1">
         <v>42200</v>
@@ -3128,7 +3104,7 @@
         <v>80.5</v>
       </c>
       <c r="F75" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G75">
         <v>5.16</v>
@@ -3139,7 +3115,7 @@
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B76" s="1">
         <v>42200</v>
@@ -3154,7 +3130,7 @@
         <v>90.6</v>
       </c>
       <c r="F76" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G76">
         <v>6.15</v>
@@ -3165,7 +3141,7 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B77" s="1">
         <v>42200</v>
@@ -3180,7 +3156,7 @@
         <v>83.7</v>
       </c>
       <c r="F77" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G77">
         <v>5.82</v>
@@ -3191,7 +3167,7 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B78" s="1">
         <v>42200</v>
@@ -3206,7 +3182,7 @@
         <v>91.9</v>
       </c>
       <c r="F78" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G78">
         <v>6.35</v>
@@ -3217,7 +3193,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B79" s="1">
         <v>42200</v>
@@ -3232,7 +3208,7 @@
         <v>90.6</v>
       </c>
       <c r="F79" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G79">
         <v>5.86</v>
@@ -3258,7 +3234,7 @@
         <v>63.1</v>
       </c>
       <c r="F80" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G80">
         <v>4.53</v>
@@ -3284,7 +3260,7 @@
         <v>75.3</v>
       </c>
       <c r="F81" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G81">
         <v>3.87</v>
@@ -3295,7 +3271,7 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B82" s="1">
         <v>42200</v>
@@ -3310,7 +3286,7 @@
         <v>80</v>
       </c>
       <c r="F82" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G82">
         <v>4.8899999999999997</v>
@@ -3362,7 +3338,7 @@
         <v>69.5</v>
       </c>
       <c r="F84" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G84">
         <v>4.34</v>
@@ -3388,7 +3364,7 @@
         <v>32.200000000000003</v>
       </c>
       <c r="F85" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G85">
         <v>2.6579999999999999</v>
@@ -3414,7 +3390,7 @@
         <v>28.3</v>
       </c>
       <c r="F86" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G86">
         <v>1.9430000000000001</v>
@@ -3440,7 +3416,7 @@
         <v>31.8</v>
       </c>
       <c r="F87" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G87">
         <v>2.79</v>
@@ -3466,7 +3442,7 @@
         <v>24.7</v>
       </c>
       <c r="F88" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G88">
         <v>1.9370000000000001</v>
@@ -3492,7 +3468,7 @@
         <v>25.4</v>
       </c>
       <c r="F89" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G89">
         <v>1.8069999999999999</v>
@@ -3518,7 +3494,7 @@
         <v>25.7</v>
       </c>
       <c r="F90" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G90">
         <v>2.5659999999999998</v>
@@ -3544,7 +3520,7 @@
         <v>27.5</v>
       </c>
       <c r="F91" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G91">
         <v>2.3650000000000002</v>
@@ -3570,7 +3546,7 @@
         <v>24.9</v>
       </c>
       <c r="F92" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G92">
         <v>2.1019999999999999</v>
@@ -3596,7 +3572,7 @@
         <v>23.9</v>
       </c>
       <c r="F93" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="G93">
         <v>0.39700000000000002</v>
@@ -3622,7 +3598,7 @@
         <v>23.9</v>
       </c>
       <c r="F94" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="G94">
         <v>2.1869999999999998</v>
@@ -3648,7 +3624,7 @@
         <v>22</v>
       </c>
       <c r="F95" t="s">
-        <v>242</v>
+        <v>221</v>
       </c>
       <c r="G95">
         <v>-1.6879999999999999</v>
@@ -3674,7 +3650,7 @@
         <v>21.7</v>
       </c>
       <c r="F96" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G96">
         <v>2.2229999999999999</v>
@@ -3700,7 +3676,7 @@
         <v>44.9</v>
       </c>
       <c r="F97" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G97">
         <v>1.1200000000000001</v>
@@ -3726,7 +3702,7 @@
         <v>30.2</v>
       </c>
       <c r="F98" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G98">
         <v>2.3170000000000002</v>
@@ -3752,7 +3728,7 @@
         <v>42.1</v>
       </c>
       <c r="F99" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G99">
         <v>2.524</v>
@@ -3763,7 +3739,7 @@
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B100" s="1">
         <v>42267</v>
@@ -3778,7 +3754,7 @@
         <v>26.6</v>
       </c>
       <c r="F100" t="s">
-        <v>242</v>
+        <v>221</v>
       </c>
       <c r="G100">
         <v>0.35299999999999998</v>
@@ -3804,7 +3780,7 @@
         <v>28.7</v>
       </c>
       <c r="F101" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G101">
         <v>2.4700000000000002</v>
@@ -3830,7 +3806,7 @@
         <v>29.3</v>
       </c>
       <c r="F102" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G102">
         <v>1.7290000000000001</v>
@@ -3856,7 +3832,7 @@
         <v>38.299999999999997</v>
       </c>
       <c r="F103" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G103">
         <v>2.96</v>
@@ -3882,7 +3858,7 @@
         <v>41.8</v>
       </c>
       <c r="F104" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G104">
         <v>2.9649999999999999</v>
@@ -3908,7 +3884,7 @@
         <v>27.6</v>
       </c>
       <c r="F105" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G105">
         <v>1.65</v>
@@ -3934,7 +3910,7 @@
         <v>31.3</v>
       </c>
       <c r="F106" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G106">
         <v>2.895</v>
@@ -3960,7 +3936,7 @@
         <v>46.6</v>
       </c>
       <c r="F107" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G107">
         <v>3.9380000000000002</v>
@@ -3986,7 +3962,7 @@
         <v>45.3</v>
       </c>
       <c r="F108" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="G108">
         <v>5.4809999999999999</v>
@@ -4012,7 +3988,7 @@
         <v>52.9</v>
       </c>
       <c r="F109" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G109">
         <v>2.59</v>
@@ -4038,7 +4014,7 @@
         <v>52.8</v>
       </c>
       <c r="F110" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G110">
         <v>3.911</v>
@@ -4064,7 +4040,7 @@
         <v>52.9</v>
       </c>
       <c r="F111" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G111">
         <v>3.6320000000000001</v>
@@ -4090,7 +4066,7 @@
         <v>45.4</v>
       </c>
       <c r="F112" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G112">
         <v>2.3959999999999999</v>
@@ -4116,7 +4092,7 @@
         <v>48</v>
       </c>
       <c r="F113" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G113">
         <v>2.851</v>
@@ -4142,7 +4118,7 @@
         <v>48.4</v>
       </c>
       <c r="F114" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G114">
         <v>2.8279999999999998</v>
@@ -4168,7 +4144,7 @@
         <v>41</v>
       </c>
       <c r="F115" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G115">
         <v>2.7719999999999998</v>
@@ -4194,7 +4170,7 @@
         <v>45.6</v>
       </c>
       <c r="F116" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G116">
         <v>2.9060000000000001</v>
@@ -4220,7 +4196,7 @@
         <v>114</v>
       </c>
       <c r="F117" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G117">
         <v>3.456</v>
@@ -4246,7 +4222,7 @@
         <v>110.9</v>
       </c>
       <c r="F118" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G118">
         <v>2.8460000000000001</v>
@@ -4272,7 +4248,7 @@
         <v>116.3</v>
       </c>
       <c r="F119" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G119">
         <v>3.3620000000000001</v>
@@ -4298,7 +4274,7 @@
         <v>122.6</v>
       </c>
       <c r="F120" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G120">
         <v>3.0529999999999999</v>
@@ -4324,7 +4300,7 @@
         <v>106.2</v>
       </c>
       <c r="F121" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G121">
         <v>2.669</v>
@@ -4350,7 +4326,7 @@
         <v>115.4</v>
       </c>
       <c r="F122" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G122">
         <v>3.3929999999999998</v>
@@ -4376,7 +4352,7 @@
         <v>126.9</v>
       </c>
       <c r="F123" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G123">
         <v>3.6579999999999999</v>
@@ -4402,7 +4378,7 @@
         <v>121.8</v>
       </c>
       <c r="F124" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="G124">
         <v>5.5179999999999998</v>
@@ -4428,7 +4404,7 @@
         <v>123.8</v>
       </c>
       <c r="F125" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G125">
         <v>3.3149999999999999</v>
@@ -4454,7 +4430,7 @@
         <v>55.7</v>
       </c>
       <c r="F126" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="G126">
         <v>5.141</v>
@@ -4480,7 +4456,7 @@
         <v>55.7</v>
       </c>
       <c r="F127" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="G127">
         <v>5.4210000000000003</v>
@@ -4506,7 +4482,7 @@
         <v>55.9</v>
       </c>
       <c r="F128" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G128">
         <v>4.7190000000000003</v>
@@ -4532,7 +4508,7 @@
         <v>55.9</v>
       </c>
       <c r="F129" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="G129">
         <v>4.96</v>
@@ -4558,7 +4534,7 @@
         <v>56.7</v>
       </c>
       <c r="F130" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G130">
         <v>4.6970000000000001</v>
@@ -4584,7 +4560,7 @@
         <v>55.2</v>
       </c>
       <c r="F131" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G131">
         <v>3.8109999999999999</v>
@@ -4610,7 +4586,7 @@
         <v>55.7</v>
       </c>
       <c r="F132" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G132">
         <v>3.3780000000000001</v>
@@ -4636,7 +4612,7 @@
         <v>54.6</v>
       </c>
       <c r="F133" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G133">
         <v>3.4079999999999999</v>
@@ -4662,7 +4638,7 @@
         <v>55.8</v>
       </c>
       <c r="F134" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="G134">
         <v>3.4609999999999999</v>
@@ -4688,7 +4664,7 @@
         <v>46.2</v>
       </c>
       <c r="F135" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G135">
         <v>3.379</v>
@@ -4714,7 +4690,7 @@
         <v>47</v>
       </c>
       <c r="F136" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="G136">
         <v>2.94</v>
@@ -4740,7 +4716,7 @@
         <v>50</v>
       </c>
       <c r="F137" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G137">
         <v>3.18</v>
@@ -4766,7 +4742,7 @@
         <v>46.6</v>
       </c>
       <c r="F138" t="s">
-        <v>245</v>
+        <v>212</v>
       </c>
       <c r="G138">
         <v>3.0979999999999999</v>
@@ -4792,7 +4768,7 @@
         <v>18</v>
       </c>
       <c r="F139" s="6" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G139" s="6">
         <v>1.0059041900000001</v>
@@ -4803,7 +4779,7 @@
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A140" s="5" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="B140" s="6">
         <v>2022</v>
@@ -4829,16 +4805,16 @@
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A141" s="5" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="B141" s="6">
         <v>2022</v>
       </c>
       <c r="C141" s="6">
-        <v>55.514560000000003</v>
+        <v>55.512961699999998</v>
       </c>
       <c r="D141" s="6">
-        <v>-5.0578782999999996</v>
+        <v>-5.0589199999999996</v>
       </c>
       <c r="E141" s="6">
         <v>12</v>
@@ -4847,394 +4823,394 @@
         <v>209</v>
       </c>
       <c r="G141" s="6">
-        <v>-1.2381</v>
+        <v>-1.0941059</v>
       </c>
       <c r="H141" s="6">
-        <v>-1.2502800000000001</v>
+        <v>-1.1420136999999999</v>
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A142" s="5" t="s">
-        <v>222</v>
+        <v>148</v>
       </c>
       <c r="B142" s="6">
         <v>2022</v>
       </c>
       <c r="C142" s="6">
-        <v>55.512961699999998</v>
+        <v>55.511519999999997</v>
       </c>
       <c r="D142" s="6">
-        <v>-5.0589199999999996</v>
+        <v>-5.0604383000000004</v>
       </c>
       <c r="E142" s="6">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="G142" s="6">
-        <v>-1.0941059</v>
+        <v>-0.8772681</v>
       </c>
       <c r="H142" s="6">
-        <v>-1.1420136999999999</v>
+        <v>-0.89055209999999996</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A143" s="5" t="s">
-        <v>223</v>
+        <v>149</v>
       </c>
       <c r="B143" s="6">
         <v>2022</v>
       </c>
       <c r="C143" s="6">
-        <v>55.512961699999998</v>
+        <v>55.509785000000001</v>
       </c>
       <c r="D143" s="6">
-        <v>-5.0589199999999996</v>
+        <v>-5.0618049999999997</v>
       </c>
       <c r="E143" s="6">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F143" s="6" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="G143" s="6">
-        <v>-1.0941059</v>
+        <v>-0.93328339999999999</v>
       </c>
       <c r="H143" s="6">
-        <v>-1.1420136999999999</v>
+        <v>-0.91669650000000003</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A144" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B144" s="6">
         <v>2022</v>
       </c>
       <c r="C144" s="6">
-        <v>55.511519999999997</v>
+        <v>55.508310000000002</v>
       </c>
       <c r="D144" s="6">
-        <v>-5.0604383000000004</v>
+        <v>-5.0619082999999998</v>
       </c>
       <c r="E144" s="6">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F144" s="6" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G144" s="6">
-        <v>-0.8772681</v>
+        <v>-0.68437999999999999</v>
       </c>
       <c r="H144" s="6">
-        <v>-0.89055209999999996</v>
+        <v>-2.2599999999999999E-2</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A145" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B145" s="6">
         <v>2022</v>
       </c>
       <c r="C145" s="6">
-        <v>55.509785000000001</v>
+        <v>55.506021699999998</v>
       </c>
       <c r="D145" s="6">
-        <v>-5.0618049999999997</v>
+        <v>-5.0631867000000002</v>
       </c>
       <c r="E145" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F145" s="6" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="G145" s="6">
-        <v>-0.93328339999999999</v>
+        <v>0.51677717000000001</v>
       </c>
       <c r="H145" s="6">
-        <v>-0.91669650000000003</v>
+        <v>1.3933649699999999</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A146" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B146" s="6">
         <v>2022</v>
       </c>
       <c r="C146" s="6">
-        <v>55.508310000000002</v>
+        <v>55.509943300000003</v>
       </c>
       <c r="D146" s="6">
-        <v>-5.0619082999999998</v>
+        <v>-5.0668882999999996</v>
       </c>
       <c r="E146" s="6">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F146" s="6" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="G146" s="6">
-        <v>-0.68437999999999999</v>
+        <v>-1.44712</v>
       </c>
       <c r="H146" s="6">
-        <v>-2.2599999999999999E-2</v>
+        <v>-1.5696600000000001</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A147" s="5" t="s">
-        <v>151</v>
+        <v>200</v>
       </c>
       <c r="B147" s="6">
         <v>2022</v>
       </c>
       <c r="C147" s="6">
-        <v>55.506021699999998</v>
+        <v>55.627719999999997</v>
       </c>
       <c r="D147" s="6">
-        <v>-5.0631867000000002</v>
+        <v>-5.1319999999999997</v>
       </c>
       <c r="E147" s="6">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F147" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G147" s="6">
-        <v>0.51677717000000001</v>
+        <v>-2.2245746999999998</v>
       </c>
       <c r="H147" s="6">
-        <v>1.3933649699999999</v>
+        <v>-1.9718081000000001</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A148" s="5" t="s">
-        <v>152</v>
+        <v>201</v>
       </c>
       <c r="B148" s="6">
         <v>2022</v>
       </c>
       <c r="C148" s="6">
-        <v>55.509943300000003</v>
+        <v>55.629108299999999</v>
       </c>
       <c r="D148" s="6">
-        <v>-5.0668882999999996</v>
+        <v>-5.1324966999999999</v>
       </c>
       <c r="E148" s="6">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F148" s="6" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="G148" s="6">
-        <v>-1.44712</v>
+        <v>-2.1023000000000001</v>
       </c>
       <c r="H148" s="6">
-        <v>-1.5696600000000001</v>
+        <v>-2.0320200000000002</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A149" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B149" s="6">
         <v>2022</v>
       </c>
       <c r="C149" s="6">
-        <v>55.627719999999997</v>
+        <v>55.628450000000001</v>
       </c>
       <c r="D149" s="6">
-        <v>-5.1319999999999997</v>
+        <v>-5.1312267</v>
       </c>
       <c r="E149" s="6">
-        <v>9</v>
-      </c>
-      <c r="F149" s="6" t="s">
-        <v>209</v>
+        <v>24</v>
+      </c>
+      <c r="F149" t="s">
+        <v>210</v>
       </c>
       <c r="G149" s="6">
-        <v>-2.2245746999999998</v>
+        <v>1.765882</v>
       </c>
       <c r="H149" s="6">
-        <v>-1.9718081000000001</v>
+        <v>1.445994</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A150" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B150" s="6">
         <v>2022</v>
       </c>
       <c r="C150" s="6">
-        <v>55.629108299999999</v>
+        <v>55.624310000000001</v>
       </c>
       <c r="D150" s="6">
-        <v>-5.1324966999999999</v>
+        <v>-5.1296483000000004</v>
       </c>
       <c r="E150" s="6">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F150" s="6" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G150" s="6">
-        <v>-2.1023000000000001</v>
+        <v>-0.2332024</v>
       </c>
       <c r="H150" s="6">
-        <v>-2.0320200000000002</v>
+        <v>0.83038142000000004</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A151" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B151" s="6">
         <v>2022</v>
       </c>
       <c r="C151" s="6">
-        <v>55.628450000000001</v>
+        <v>55.620741700000004</v>
       </c>
       <c r="D151" s="6">
-        <v>-5.1312267</v>
+        <v>-5.1286649999999998</v>
       </c>
       <c r="E151" s="6">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F151" s="6" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="G151" s="6">
-        <v>1.765882</v>
+        <v>-1.7215138000000001</v>
       </c>
       <c r="H151" s="6">
-        <v>1.445994</v>
+        <v>-2.0978943999999999</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A152" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B152" s="6">
         <v>2022</v>
       </c>
       <c r="C152" s="6">
-        <v>55.624310000000001</v>
+        <v>55.618588299999999</v>
       </c>
       <c r="D152" s="6">
-        <v>-5.1296483000000004</v>
+        <v>-5.1272282999999996</v>
       </c>
       <c r="E152" s="6">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F152" s="6" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
       <c r="G152" s="6">
-        <v>-0.2332024</v>
+        <v>2.5678380000000001</v>
       </c>
       <c r="H152" s="6">
-        <v>0.83038142000000004</v>
+        <v>3.1196980000000001</v>
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A153" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B153" s="6">
         <v>2022</v>
       </c>
       <c r="C153" s="6">
-        <v>55.620741700000004</v>
+        <v>55.616418299999999</v>
       </c>
       <c r="D153" s="6">
-        <v>-5.1286649999999998</v>
+        <v>-5.1272450000000003</v>
       </c>
       <c r="E153" s="6">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F153" s="6" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G153" s="6">
-        <v>-1.7215138000000001</v>
+        <v>-0.56488000000000005</v>
       </c>
       <c r="H153" s="6">
-        <v>-2.0978943999999999</v>
+        <v>0.59134399999999998</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A154" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B154" s="6">
         <v>2022</v>
       </c>
       <c r="C154" s="6">
-        <v>55.618588299999999</v>
+        <v>55.610424999999999</v>
       </c>
       <c r="D154" s="6">
-        <v>-5.1272282999999996</v>
+        <v>-5.1223466999999996</v>
       </c>
       <c r="E154" s="6">
         <v>22</v>
       </c>
       <c r="F154" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G154" s="6">
-        <v>2.5678380000000001</v>
+        <v>2.21485618</v>
       </c>
       <c r="H154" s="6">
-        <v>3.1196980000000001</v>
+        <v>2.78901281</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A155" s="5" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B155" s="6">
         <v>2022</v>
       </c>
       <c r="C155" s="6">
-        <v>55.616418299999999</v>
+        <v>55.608693299999999</v>
       </c>
       <c r="D155" s="6">
-        <v>-5.1272450000000003</v>
+        <v>-5.1249750000000001</v>
       </c>
       <c r="E155" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F155" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G155" s="6">
-        <v>-0.56488000000000005</v>
+        <v>2.21485618</v>
       </c>
       <c r="H155" s="6">
-        <v>0.59134399999999998</v>
+        <v>2.78901281</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A156" s="5" t="s">
-        <v>207</v>
+        <v>238</v>
       </c>
       <c r="B156" s="6">
         <v>2022</v>
       </c>
       <c r="C156" s="6">
-        <v>55.610424999999999</v>
+        <v>55.608693299999999</v>
       </c>
       <c r="D156" s="6">
-        <v>-5.1223466999999996</v>
+        <v>-5.1249750000000001</v>
       </c>
       <c r="E156" s="6">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F156" s="6" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="G156" s="6">
         <v>2.21485618</v>
@@ -5245,1938 +5221,1892 @@
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A157" s="5" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="B157" s="6">
         <v>2022</v>
       </c>
       <c r="C157" s="6">
-        <v>55.608693299999999</v>
+        <v>55.605878300000001</v>
       </c>
       <c r="D157" s="6">
-        <v>-5.1249750000000001</v>
+        <v>-5.1222383000000002</v>
       </c>
       <c r="E157" s="6">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F157" s="6" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="G157" s="6">
-        <v>2.21485618</v>
+        <v>2.3442729999999998</v>
       </c>
       <c r="H157" s="6">
-        <v>2.78901281</v>
+        <v>2.3343259999999999</v>
       </c>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A158" s="5" t="s">
-        <v>248</v>
+        <v>188</v>
       </c>
       <c r="B158" s="6">
         <v>2022</v>
       </c>
       <c r="C158" s="6">
-        <v>55.608693299999999</v>
+        <v>55.435301699999997</v>
       </c>
       <c r="D158" s="6">
-        <v>-5.1249750000000001</v>
+        <v>-5.3061499999999997</v>
       </c>
       <c r="E158" s="6">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F158" s="6" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G158" s="6">
-        <v>2.21485618</v>
+        <v>0.59241641</v>
       </c>
       <c r="H158" s="6">
-        <v>2.78901281</v>
+        <v>0.84917187000000005</v>
       </c>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A159" s="5" t="s">
-        <v>208</v>
+        <v>187</v>
       </c>
       <c r="B159" s="6">
         <v>2022</v>
       </c>
       <c r="C159" s="6">
-        <v>55.605878300000001</v>
+        <v>55.428044999999997</v>
       </c>
       <c r="D159" s="6">
-        <v>-5.1222383000000002</v>
+        <v>-5.2885666999999996</v>
       </c>
       <c r="E159" s="6">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F159" s="6" t="s">
         <v>211</v>
       </c>
       <c r="G159" s="6">
-        <v>2.3442729999999998</v>
+        <v>2.08641706</v>
       </c>
       <c r="H159" s="6">
-        <v>2.3343259999999999</v>
+        <v>2.7133886500000002</v>
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A160" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B160" s="6">
         <v>2022</v>
       </c>
       <c r="C160" s="6">
-        <v>55.435301699999997</v>
+        <v>55.429683300000001</v>
       </c>
       <c r="D160" s="6">
-        <v>-5.3061499999999997</v>
+        <v>-5.30593</v>
       </c>
       <c r="E160" s="6">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F160" s="6" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="G160" s="6">
-        <v>0.59241641</v>
+        <v>1.5488489999999999</v>
       </c>
       <c r="H160" s="6">
-        <v>0.84917187000000005</v>
+        <v>2.099818</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A161" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B161" s="6">
         <v>2022</v>
       </c>
       <c r="C161" s="6">
-        <v>55.428044999999997</v>
+        <v>55.425579999999997</v>
       </c>
       <c r="D161" s="6">
-        <v>-5.2885666999999996</v>
+        <v>-5.2963766999999997</v>
       </c>
       <c r="E161" s="6">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F161" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G161" s="6">
-        <v>2.08641706</v>
+        <v>1.3355805199999999</v>
       </c>
       <c r="H161" s="6">
-        <v>2.7133886500000002</v>
+        <v>1.2567770599999999</v>
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A162" s="5" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B162" s="6">
         <v>2022</v>
       </c>
       <c r="C162" s="6">
-        <v>55.429683300000001</v>
+        <v>55.423270000000002</v>
       </c>
       <c r="D162" s="6">
-        <v>-5.30593</v>
+        <v>-5.3063617000000001</v>
       </c>
       <c r="E162" s="6">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F162" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G162" s="6">
-        <v>1.5488489999999999</v>
+        <v>1.89480388</v>
       </c>
       <c r="H162" s="6">
-        <v>2.099818</v>
+        <v>1.88817729</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A163" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B163" s="6">
         <v>2022</v>
       </c>
       <c r="C163" s="6">
-        <v>55.425579999999997</v>
+        <v>55.4238517</v>
       </c>
       <c r="D163" s="6">
-        <v>-5.2963766999999997</v>
+        <v>-5.2959867000000003</v>
       </c>
       <c r="E163" s="6">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F163" s="6" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="G163" s="6">
-        <v>1.3355805199999999</v>
+        <v>1.5321192800000001</v>
       </c>
       <c r="H163" s="6">
-        <v>1.2567770599999999</v>
+        <v>0.98185339999999999</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A164" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B164" s="6">
         <v>2022</v>
       </c>
       <c r="C164" s="6">
-        <v>55.423270000000002</v>
+        <v>55.421651699999998</v>
       </c>
       <c r="D164" s="6">
-        <v>-5.3063617000000001</v>
+        <v>-5.2880482999999998</v>
       </c>
       <c r="E164" s="6">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F164" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G164" s="6">
-        <v>1.89480388</v>
+        <v>1.9910190000000001</v>
       </c>
       <c r="H164" s="6">
-        <v>1.88817729</v>
+        <v>2.0038860000000001</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A165" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B165" s="6">
         <v>2022</v>
       </c>
       <c r="C165" s="6">
-        <v>55.4238517</v>
+        <v>55.420043300000003</v>
       </c>
       <c r="D165" s="6">
-        <v>-5.2959867000000003</v>
+        <v>-5.3021117000000002</v>
       </c>
       <c r="E165" s="6">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F165" s="6" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="G165" s="6">
-        <v>1.5321192800000001</v>
+        <v>2.3229115400000002</v>
       </c>
       <c r="H165" s="6">
-        <v>0.98185339999999999</v>
+        <v>2.8630046999999998</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A166" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B166" s="6">
         <v>2022</v>
       </c>
       <c r="C166" s="6">
-        <v>55.421651699999998</v>
+        <v>55.419975000000001</v>
       </c>
       <c r="D166" s="6">
-        <v>-5.2880482999999998</v>
+        <v>-5.2994317000000004</v>
       </c>
       <c r="E166" s="6">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F166" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G166" s="6">
-        <v>1.9910190000000001</v>
+        <v>1.2403518499999999</v>
       </c>
       <c r="H166" s="6">
-        <v>2.0038860000000001</v>
+        <v>1.82353421</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A167" s="5" t="s">
-        <v>181</v>
+        <v>139</v>
       </c>
       <c r="B167" s="6">
         <v>2022</v>
       </c>
       <c r="C167" s="6">
-        <v>55.420043300000003</v>
+        <v>55.543558300000001</v>
       </c>
       <c r="D167" s="6">
-        <v>-5.3021117000000002</v>
+        <v>-5.0838482999999997</v>
       </c>
       <c r="E167" s="6">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F167" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G167" s="6">
-        <v>2.3229115400000002</v>
+        <v>0.33536194000000003</v>
       </c>
       <c r="H167" s="6">
-        <v>2.8630046999999998</v>
+        <v>1.24935062</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A168" s="5" t="s">
-        <v>180</v>
+        <v>138</v>
       </c>
       <c r="B168" s="6">
         <v>2022</v>
       </c>
       <c r="C168" s="6">
-        <v>55.419975000000001</v>
+        <v>55.542693300000003</v>
       </c>
       <c r="D168" s="6">
-        <v>-5.2994317000000004</v>
+        <v>-5.0818300000000001</v>
       </c>
       <c r="E168" s="6">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F168" s="6" t="s">
         <v>210</v>
       </c>
       <c r="G168" s="6">
-        <v>1.2403518499999999</v>
+        <v>1.3273678099999999</v>
       </c>
       <c r="H168" s="6">
-        <v>1.82353421</v>
+        <v>1.71973262</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A169" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B169" s="6">
         <v>2022</v>
       </c>
       <c r="C169" s="6">
-        <v>55.543558300000001</v>
+        <v>55.542906700000003</v>
       </c>
       <c r="D169" s="6">
-        <v>-5.0838482999999997</v>
+        <v>-5.0781799999999997</v>
       </c>
       <c r="E169" s="6">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F169" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G169" s="6">
-        <v>0.33536194000000003</v>
+        <v>2.29970856</v>
       </c>
       <c r="H169" s="6">
-        <v>1.24935062</v>
+        <v>2.32652021</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A170" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B170" s="6">
         <v>2022</v>
       </c>
       <c r="C170" s="6">
-        <v>55.542693300000003</v>
+        <v>55.540925000000001</v>
       </c>
       <c r="D170" s="6">
-        <v>-5.0818300000000001</v>
+        <v>-5.0808767000000001</v>
       </c>
       <c r="E170" s="6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F170" s="6" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="G170" s="6">
-        <v>1.3273678099999999</v>
+        <v>0.85499283000000004</v>
       </c>
       <c r="H170" s="6">
-        <v>1.71973262</v>
+        <v>0.72702155000000002</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A171" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B171" s="6">
         <v>2022</v>
       </c>
       <c r="C171" s="6">
-        <v>55.542906700000003</v>
+        <v>55.539998300000001</v>
       </c>
       <c r="D171" s="6">
-        <v>-5.0781799999999997</v>
+        <v>-5.0787800000000001</v>
       </c>
       <c r="E171" s="6">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F171" s="6" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="G171" s="6">
-        <v>2.29970856</v>
+        <v>-0.9167497</v>
       </c>
       <c r="H171" s="6">
-        <v>2.32652021</v>
+        <v>-0.94227070000000002</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A172" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B172" s="6">
         <v>2022</v>
       </c>
       <c r="C172" s="6">
-        <v>55.540925000000001</v>
+        <v>55.539498299999998</v>
       </c>
       <c r="D172" s="6">
-        <v>-5.0808767000000001</v>
+        <v>-5.0767499999999997</v>
       </c>
       <c r="E172" s="6">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F172" s="6" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="G172" s="6">
-        <v>0.85499283000000004</v>
+        <v>1.8336098599999999</v>
       </c>
       <c r="H172" s="6">
-        <v>0.72702155000000002</v>
+        <v>2.3796525800000001</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A173" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B173" s="6">
         <v>2022</v>
       </c>
       <c r="C173" s="6">
-        <v>55.539998300000001</v>
+        <v>55.537631699999999</v>
       </c>
       <c r="D173" s="6">
-        <v>-5.0787800000000001</v>
+        <v>-5.0753300000000001</v>
       </c>
       <c r="E173" s="6">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F173" s="6" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="G173" s="6">
-        <v>-0.9167497</v>
+        <v>2.4453309999999999</v>
       </c>
       <c r="H173" s="6">
-        <v>-0.94227070000000002</v>
+        <v>2.4670100000000001</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A174" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B174" s="6">
         <v>2022</v>
       </c>
       <c r="C174" s="6">
-        <v>55.539498299999998</v>
+        <v>55.536825</v>
       </c>
       <c r="D174" s="6">
-        <v>-5.0767499999999997</v>
+        <v>-5.0725382999999997</v>
       </c>
       <c r="E174" s="6">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F174" s="6" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="G174" s="6">
-        <v>1.8336098599999999</v>
+        <v>-1.0870347</v>
       </c>
       <c r="H174" s="6">
-        <v>2.3796525800000001</v>
+        <v>-0.99440499999999998</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A175" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B175" s="6">
         <v>2022</v>
       </c>
       <c r="C175" s="6">
-        <v>55.537631699999999</v>
+        <v>55.534611699999999</v>
       </c>
       <c r="D175" s="6">
-        <v>-5.0753300000000001</v>
+        <v>-5.0696433000000001</v>
       </c>
       <c r="E175" s="6">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F175" s="6" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="G175" s="6">
-        <v>2.4453309999999999</v>
+        <v>-0.66170479999999998</v>
       </c>
       <c r="H175" s="6">
-        <v>2.4670100000000001</v>
+        <v>-2.83967E-2</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A176" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B176" s="6">
         <v>2022</v>
       </c>
       <c r="C176" s="6">
-        <v>55.536825</v>
+        <v>55.53275</v>
       </c>
       <c r="D176" s="6">
-        <v>-5.0725382999999997</v>
+        <v>-5.0696383000000003</v>
       </c>
       <c r="E176" s="6">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F176" s="6" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="G176" s="6">
-        <v>-1.0870347</v>
+        <v>1.8002264800000001</v>
       </c>
       <c r="H176" s="6">
-        <v>-0.99440499999999998</v>
+        <v>2.2339649000000001</v>
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A177" s="5" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B177" s="6">
         <v>2022</v>
       </c>
       <c r="C177" s="6">
-        <v>55.534611699999999</v>
+        <v>55.443743300000001</v>
       </c>
       <c r="D177" s="6">
-        <v>-5.0696433000000001</v>
+        <v>-5.0937732999999996</v>
       </c>
       <c r="E177" s="6">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F177" s="6" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="G177" s="6">
-        <v>-0.66170479999999998</v>
+        <v>0.70437358999999999</v>
       </c>
       <c r="H177" s="6">
-        <v>-2.83967E-2</v>
+        <v>0.58482942000000004</v>
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A178" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B178" s="6">
         <v>2022</v>
       </c>
       <c r="C178" s="6">
-        <v>55.53275</v>
+        <v>55.440919999999998</v>
       </c>
       <c r="D178" s="6">
-        <v>-5.0696383000000003</v>
+        <v>-5.0946350000000002</v>
       </c>
       <c r="E178" s="6">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F178" s="6" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="G178" s="6">
-        <v>1.8002264800000001</v>
+        <v>-0.47783999999999999</v>
       </c>
       <c r="H178" s="6">
-        <v>2.2339649000000001</v>
+        <v>-0.42727999999999999</v>
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A179" s="5" t="s">
-        <v>153</v>
+        <v>213</v>
       </c>
       <c r="B179" s="6">
         <v>2022</v>
       </c>
       <c r="C179" s="6">
-        <v>55.443743300000001</v>
+        <v>55.438981699999999</v>
       </c>
       <c r="D179" s="6">
-        <v>-5.0937732999999996</v>
+        <v>-5.1023966999999999</v>
       </c>
       <c r="E179" s="6">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F179" s="6" t="s">
-        <v>226</v>
+        <v>209</v>
       </c>
       <c r="G179" s="6">
-        <v>0.70437358999999999</v>
+        <v>-0.87943470000000001</v>
       </c>
       <c r="H179" s="6">
-        <v>0.58482942000000004</v>
+        <v>-1.2672935999999999</v>
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A180" s="5" t="s">
-        <v>154</v>
+        <v>214</v>
       </c>
       <c r="B180" s="6">
         <v>2022</v>
       </c>
       <c r="C180" s="6">
-        <v>55.440919999999998</v>
+        <v>55.438981699999999</v>
       </c>
       <c r="D180" s="6">
-        <v>-5.0946350000000002</v>
+        <v>-5.1023966999999999</v>
       </c>
       <c r="E180" s="6">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F180" s="6" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="G180" s="6">
-        <v>-0.47783999999999999</v>
+        <v>-0.87943470000000001</v>
       </c>
       <c r="H180" s="6">
-        <v>-0.42727999999999999</v>
+        <v>-1.2672935999999999</v>
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A181" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B181" s="6">
         <v>2022</v>
       </c>
       <c r="C181" s="6">
-        <v>55.438981699999999</v>
+        <v>55.439728299999999</v>
       </c>
       <c r="D181" s="6">
-        <v>-5.1023966999999999</v>
+        <v>-5.0974233</v>
       </c>
       <c r="E181" s="6">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F181" s="6" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="G181" s="6">
-        <v>-0.87943470000000001</v>
+        <v>-0.70383260000000003</v>
       </c>
       <c r="H181" s="6">
-        <v>-1.2672935999999999</v>
+        <v>-0.68010870000000001</v>
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A182" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B182" s="6">
         <v>2022</v>
       </c>
       <c r="C182" s="6">
-        <v>55.438981699999999</v>
+        <v>55.439728299999999</v>
       </c>
       <c r="D182" s="6">
-        <v>-5.1023966999999999</v>
+        <v>-5.0974233</v>
       </c>
       <c r="E182" s="6">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F182" s="6" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="G182" s="6">
-        <v>-0.87943470000000001</v>
+        <v>-0.70383260000000003</v>
       </c>
       <c r="H182" s="6">
-        <v>-1.2672935999999999</v>
+        <v>-0.68010870000000001</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A183" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B183" s="6">
         <v>2022</v>
       </c>
       <c r="C183" s="6">
-        <v>55.439728299999999</v>
+        <v>55.436023300000002</v>
       </c>
       <c r="D183" s="6">
-        <v>-5.0974233</v>
+        <v>-5.1054917</v>
       </c>
       <c r="E183" s="6">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F183" s="6" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="G183" s="6">
-        <v>-0.70383260000000003</v>
+        <v>-1.3550135999999999</v>
       </c>
       <c r="H183" s="6">
-        <v>-0.68010870000000001</v>
+        <v>-1.3941920000000001</v>
       </c>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A184" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B184" s="6">
         <v>2022</v>
       </c>
       <c r="C184" s="6">
-        <v>55.439728299999999</v>
+        <v>55.436023300000002</v>
       </c>
       <c r="D184" s="6">
-        <v>-5.0974233</v>
+        <v>-5.1054917</v>
       </c>
       <c r="E184" s="6">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F184" s="6" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="G184" s="6">
-        <v>-0.70383260000000003</v>
+        <v>-1.3550135999999999</v>
       </c>
       <c r="H184" s="6">
-        <v>-0.68010870000000001</v>
+        <v>-1.3941920000000001</v>
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A185" s="5" t="s">
-        <v>217</v>
+        <v>165</v>
       </c>
       <c r="B185" s="6">
         <v>2022</v>
       </c>
       <c r="C185" s="6">
-        <v>55.436023300000002</v>
+        <v>55.432773300000001</v>
       </c>
       <c r="D185" s="6">
-        <v>-5.1054917</v>
+        <v>-5.1058899999999996</v>
       </c>
       <c r="E185" s="6">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F185" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G185" s="6">
-        <v>-1.3550135999999999</v>
+        <v>2.5983779999999999</v>
       </c>
       <c r="H185" s="6">
-        <v>-1.3941920000000001</v>
+        <v>2.6431200000000001</v>
       </c>
     </row>
     <row r="186" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A186" s="5" t="s">
-        <v>218</v>
+        <v>166</v>
       </c>
       <c r="B186" s="6">
         <v>2022</v>
       </c>
       <c r="C186" s="6">
-        <v>55.436023300000002</v>
+        <v>55.432441699999998</v>
       </c>
       <c r="D186" s="6">
-        <v>-5.1054917</v>
+        <v>-5.1093000000000002</v>
       </c>
       <c r="E186" s="6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F186" s="6" t="s">
         <v>209</v>
       </c>
       <c r="G186" s="6">
-        <v>-1.3550135999999999</v>
+        <v>-1.48515</v>
       </c>
       <c r="H186" s="6">
-        <v>-1.3941920000000001</v>
+        <v>-1.69095</v>
       </c>
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A187" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B187" s="6">
         <v>2022</v>
       </c>
       <c r="C187" s="6">
-        <v>55.432773300000001</v>
+        <v>55.429090000000002</v>
       </c>
       <c r="D187" s="6">
-        <v>-5.1058899999999996</v>
+        <v>-5.1041582999999999</v>
       </c>
       <c r="E187" s="6">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F187" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G187" s="6">
-        <v>2.5983779999999999</v>
+        <v>2.1758890000000002</v>
       </c>
       <c r="H187" s="6">
-        <v>2.6431200000000001</v>
+        <v>1.886816</v>
       </c>
     </row>
     <row r="188" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A188" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B188" s="6">
         <v>2022</v>
       </c>
       <c r="C188" s="6">
-        <v>55.432441699999998</v>
+        <v>55.428848299999999</v>
       </c>
       <c r="D188" s="6">
-        <v>-5.1093000000000002</v>
+        <v>-5.1089399999999996</v>
       </c>
       <c r="E188" s="6">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F188" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G188" s="6">
-        <v>-1.48515</v>
+        <v>2.0723796800000001</v>
       </c>
       <c r="H188" s="6">
-        <v>-1.69095</v>
+        <v>1.84313639</v>
       </c>
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A189" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B189" s="6">
         <v>2022</v>
       </c>
       <c r="C189" s="6">
-        <v>55.429090000000002</v>
+        <v>55.428778299999998</v>
       </c>
       <c r="D189" s="6">
-        <v>-5.1041582999999999</v>
+        <v>-5.1117667000000004</v>
       </c>
       <c r="E189" s="6">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F189" s="6" t="s">
         <v>210</v>
       </c>
       <c r="G189" s="6">
-        <v>2.1758890000000002</v>
+        <v>2.31374485</v>
       </c>
       <c r="H189" s="6">
-        <v>1.886816</v>
+        <v>1.6482166300000001</v>
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A190" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="B190" s="6">
-        <v>2022</v>
-      </c>
-      <c r="C190" s="6">
-        <v>55.428848299999999</v>
-      </c>
-      <c r="D190" s="6">
-        <v>-5.1089399999999996</v>
-      </c>
-      <c r="E190" s="6">
-        <v>26</v>
+      <c r="A190" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B190" s="8">
+        <v>2022</v>
+      </c>
+      <c r="C190" s="8">
+        <v>55.578164999999998</v>
+      </c>
+      <c r="D190" s="8">
+        <v>-5.0751217000000004</v>
+      </c>
+      <c r="E190" s="8">
+        <v>85</v>
       </c>
       <c r="F190" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="G190" s="6">
-        <v>2.0723796800000001</v>
-      </c>
-      <c r="H190" s="6">
-        <v>1.84313639</v>
+        <v>223</v>
+      </c>
+      <c r="G190" s="8">
+        <v>4.9221149999999998</v>
+      </c>
+      <c r="H190" s="8">
+        <v>4.7988479999999996</v>
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A191" s="5" t="s">
-        <v>169</v>
+        <v>131</v>
       </c>
       <c r="B191" s="6">
         <v>2022</v>
       </c>
       <c r="C191" s="6">
-        <v>55.428778299999998</v>
+        <v>55.575746700000003</v>
       </c>
       <c r="D191" s="6">
-        <v>-5.1117667000000004</v>
+        <v>-5.0634217000000001</v>
       </c>
       <c r="E191" s="6">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="F191" s="6" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="G191" s="6">
-        <v>2.31374485</v>
+        <v>5.3898219999999997</v>
       </c>
       <c r="H191" s="6">
-        <v>1.6482166300000001</v>
+        <v>4.8407239999999998</v>
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A192" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="B192" s="8">
-        <v>2022</v>
-      </c>
-      <c r="C192" s="8">
-        <v>55.578164999999998</v>
-      </c>
-      <c r="D192" s="8">
-        <v>-5.0751217000000004</v>
-      </c>
-      <c r="E192" s="8">
-        <v>85</v>
+      <c r="A192" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B192" s="6">
+        <v>2022</v>
+      </c>
+      <c r="C192" s="6">
+        <v>55.575000000000003</v>
+      </c>
+      <c r="D192" s="6">
+        <v>-5.0676717</v>
+      </c>
+      <c r="E192" s="6">
+        <v>92</v>
       </c>
       <c r="F192" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="G192" s="8">
-        <v>4.9221149999999998</v>
-      </c>
-      <c r="H192" s="8">
-        <v>4.7988479999999996</v>
+        <v>224</v>
+      </c>
+      <c r="G192" s="6">
+        <v>5.5496970000000001</v>
+      </c>
+      <c r="H192" s="6">
+        <v>5.187379</v>
       </c>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A193" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B193" s="6">
         <v>2022</v>
       </c>
       <c r="C193" s="6">
-        <v>55.575746700000003</v>
+        <v>55.571505000000002</v>
       </c>
       <c r="D193" s="6">
-        <v>-5.0634217000000001</v>
+        <v>-5.0703266999999999</v>
       </c>
       <c r="E193" s="6">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="F193" s="6" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="G193" s="6">
-        <v>5.3898219999999997</v>
+        <v>2.8088143799999998</v>
       </c>
       <c r="H193" s="6">
-        <v>4.8407239999999998</v>
+        <v>3.5041111699999998</v>
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A194" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B194" s="6">
-        <v>2022</v>
-      </c>
-      <c r="C194" s="6">
-        <v>55.575000000000003</v>
-      </c>
-      <c r="D194" s="6">
-        <v>-5.0676717</v>
-      </c>
-      <c r="E194" s="6">
-        <v>92</v>
-      </c>
-      <c r="F194" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="G194" s="6">
-        <v>5.5496970000000001</v>
-      </c>
-      <c r="H194" s="6">
-        <v>5.187379</v>
+      <c r="A194" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B194" s="8">
+        <v>2022</v>
+      </c>
+      <c r="C194" s="8">
+        <v>55.5696133</v>
+      </c>
+      <c r="D194" s="8">
+        <v>-5.0652566999999999</v>
+      </c>
+      <c r="E194" s="8">
+        <v>76</v>
+      </c>
+      <c r="F194" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="G194" s="8">
+        <v>5.1926678700000002</v>
+      </c>
+      <c r="H194" s="8">
+        <v>4.9356857200000004</v>
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A195" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B195" s="6">
         <v>2022</v>
       </c>
       <c r="C195" s="6">
-        <v>55.571505000000002</v>
+        <v>55.578229999999998</v>
       </c>
       <c r="D195" s="6">
-        <v>-5.0703266999999999</v>
+        <v>-5.0637983000000002</v>
       </c>
       <c r="E195" s="6">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="F195" s="6" t="s">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="G195" s="6">
-        <v>2.8088143799999998</v>
+        <v>6.4273921999999999</v>
       </c>
       <c r="H195" s="6">
-        <v>3.5041111699999998</v>
+        <v>6.1208175899999997</v>
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A196" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B196" s="8">
-        <v>2022</v>
-      </c>
-      <c r="C196" s="8">
-        <v>55.5696133</v>
-      </c>
-      <c r="D196" s="8">
-        <v>-5.0652566999999999</v>
-      </c>
-      <c r="E196" s="8">
-        <v>76</v>
-      </c>
-      <c r="F196" s="8" t="s">
-        <v>227</v>
-      </c>
-      <c r="G196" s="8">
-        <v>5.1926678700000002</v>
-      </c>
-      <c r="H196" s="8">
-        <v>4.9356857200000004</v>
+      <c r="A196" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B196" s="6">
+        <v>2022</v>
+      </c>
+      <c r="C196" s="6">
+        <v>55.569665000000001</v>
+      </c>
+      <c r="D196" s="6">
+        <v>-5.0627199999999997</v>
+      </c>
+      <c r="E196" s="6">
+        <v>81</v>
+      </c>
+      <c r="F196" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G196" s="6">
+        <v>3.8201953400000002</v>
+      </c>
+      <c r="H196" s="6">
+        <v>4.2576697100000001</v>
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B197" s="6">
         <v>2022</v>
       </c>
       <c r="C197" s="6">
-        <v>55.578229999999998</v>
+        <v>55.568145000000001</v>
       </c>
       <c r="D197" s="6">
-        <v>-5.0637983000000002</v>
+        <v>-5.0546449999999998</v>
       </c>
       <c r="E197" s="6">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="F197" s="6" t="s">
-        <v>246</v>
+        <v>223</v>
       </c>
       <c r="G197" s="6">
-        <v>6.4273921999999999</v>
+        <v>3.33810691</v>
       </c>
       <c r="H197" s="6">
-        <v>6.1208175899999997</v>
+        <v>4.1829467899999999</v>
       </c>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A198" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B198" s="6">
         <v>2022</v>
       </c>
       <c r="C198" s="6">
-        <v>55.569665000000001</v>
+        <v>55.565426700000003</v>
       </c>
       <c r="D198" s="6">
-        <v>-5.0627199999999997</v>
+        <v>-5.0585966999999998</v>
       </c>
       <c r="E198" s="6">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="F198" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G198" s="6">
-        <v>3.8201953400000002</v>
+        <v>5.1315345199999998</v>
       </c>
       <c r="H198" s="6">
-        <v>4.2576697100000001</v>
+        <v>5.0327548599999998</v>
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A199" s="5" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="B199" s="6">
         <v>2022</v>
       </c>
       <c r="C199" s="6">
-        <v>55.568145000000001</v>
+        <v>55.403263299999999</v>
       </c>
       <c r="D199" s="6">
-        <v>-5.0546449999999998</v>
+        <v>-5.1829033000000004</v>
       </c>
       <c r="E199" s="6">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="F199" s="6" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="G199" s="6">
-        <v>3.33810691</v>
+        <v>3.0721539999999998</v>
       </c>
       <c r="H199" s="6">
-        <v>4.1829467899999999</v>
+        <v>3.8256009999999998</v>
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A200" s="5" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="B200" s="6">
         <v>2022</v>
       </c>
       <c r="C200" s="6">
-        <v>55.565426700000003</v>
+        <v>55.400763300000001</v>
       </c>
       <c r="D200" s="6">
-        <v>-5.0585966999999998</v>
+        <v>-5.1908583000000004</v>
       </c>
       <c r="E200" s="6">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="F200" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="G200" s="6">
-        <v>5.1315345199999998</v>
+        <v>3.3235899999999998</v>
       </c>
       <c r="H200" s="6">
-        <v>5.0327548599999998</v>
+        <v>4.1019560000000004</v>
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A201" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B201" s="6">
         <v>2022</v>
       </c>
       <c r="C201" s="6">
-        <v>55.403263299999999</v>
+        <v>55.410046700000002</v>
       </c>
       <c r="D201" s="6">
-        <v>-5.1829033000000004</v>
+        <v>-5.1906800000000004</v>
       </c>
       <c r="E201" s="6">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F201" s="6" t="s">
         <v>212</v>
       </c>
       <c r="G201" s="6">
-        <v>3.0721539999999998</v>
+        <v>3.16897027</v>
       </c>
       <c r="H201" s="6">
-        <v>3.8256009999999998</v>
+        <v>3.97923392</v>
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A202" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B202" s="6">
         <v>2022</v>
       </c>
       <c r="C202" s="6">
-        <v>55.400763300000001</v>
+        <v>55.401665000000001</v>
       </c>
       <c r="D202" s="6">
-        <v>-5.1908583000000004</v>
+        <v>-5.1971600000000002</v>
       </c>
       <c r="E202" s="6">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F202" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G202" s="6">
-        <v>3.3235899999999998</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="H202" s="6">
-        <v>4.1019560000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A203" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B203" s="6">
         <v>2022</v>
       </c>
       <c r="C203" s="6">
-        <v>55.410046700000002</v>
+        <v>55.407793300000002</v>
       </c>
       <c r="D203" s="6">
-        <v>-5.1906800000000004</v>
+        <v>-5.1866000000000003</v>
       </c>
       <c r="E203" s="6">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F203" s="6" t="s">
         <v>212</v>
       </c>
       <c r="G203" s="6">
-        <v>3.16897027</v>
+        <v>3.1529339699999999</v>
       </c>
       <c r="H203" s="6">
-        <v>3.97923392</v>
+        <v>3.95173109</v>
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A204" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B204" s="6">
         <v>2022</v>
       </c>
       <c r="C204" s="6">
-        <v>55.401665000000001</v>
+        <v>55.395856700000003</v>
       </c>
       <c r="D204" s="6">
-        <v>-5.1971600000000002</v>
+        <v>-5.1998017000000001</v>
       </c>
       <c r="E204" s="6">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F204" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G204" s="6">
-        <v>4.0999999999999996</v>
+        <v>4.6440000000000001</v>
       </c>
       <c r="H204" s="6">
-        <v>4.7</v>
+        <v>4.9560000000000004</v>
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A205" s="5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B205" s="6">
         <v>2022</v>
       </c>
       <c r="C205" s="6">
-        <v>55.407793300000002</v>
+        <v>55.396521700000001</v>
       </c>
       <c r="D205" s="6">
-        <v>-5.1866000000000003</v>
+        <v>-5.2066566999999999</v>
       </c>
       <c r="E205" s="6">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F205" s="6" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="G205" s="6">
-        <v>3.1529339699999999</v>
+        <v>4.9560000000000004</v>
       </c>
       <c r="H205" s="6">
-        <v>3.95173109</v>
+        <v>5.2519999999999998</v>
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A206" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B206" s="6">
         <v>2022</v>
       </c>
       <c r="C206" s="6">
-        <v>55.395856700000003</v>
+        <v>55.392530000000001</v>
       </c>
       <c r="D206" s="6">
-        <v>-5.1998017000000001</v>
+        <v>-5.2044183000000004</v>
       </c>
       <c r="E206" s="6">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F206" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G206" s="6">
-        <v>4.6440000000000001</v>
+        <v>5.4240000000000004</v>
       </c>
       <c r="H206" s="6">
-        <v>4.9560000000000004</v>
+        <v>5.508</v>
       </c>
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A207" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B207" s="6">
         <v>2022</v>
       </c>
       <c r="C207" s="6">
-        <v>55.396521700000001</v>
+        <v>55.393268300000003</v>
       </c>
       <c r="D207" s="6">
-        <v>-5.2066566999999999</v>
+        <v>-5.2103883</v>
       </c>
       <c r="E207" s="6">
         <v>55</v>
       </c>
       <c r="F207" s="6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G207" s="6">
-        <v>4.9560000000000004</v>
+        <v>5.3949999999999996</v>
       </c>
       <c r="H207" s="6">
-        <v>5.2519999999999998</v>
+        <v>5.5579999999999998</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A208" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B208" s="6">
         <v>2022</v>
       </c>
       <c r="C208" s="6">
-        <v>55.392530000000001</v>
+        <v>55.3937983</v>
       </c>
       <c r="D208" s="6">
-        <v>-5.2044183000000004</v>
+        <v>-5.1951200000000002</v>
       </c>
       <c r="E208" s="6">
         <v>55</v>
       </c>
       <c r="F208" s="6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G208" s="6">
-        <v>5.4240000000000004</v>
+        <v>5.1109999999999998</v>
       </c>
       <c r="H208" s="6">
-        <v>5.508</v>
+        <v>5.3239999999999998</v>
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A209" s="5" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="B209" s="6">
         <v>2022</v>
       </c>
       <c r="C209" s="6">
-        <v>55.393268300000003</v>
+        <v>55.4562217</v>
       </c>
       <c r="D209" s="6">
-        <v>-5.2103883</v>
+        <v>-5.3669700000000002</v>
       </c>
       <c r="E209" s="6">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="F209" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="G209" s="6">
-        <v>5.3949999999999996</v>
+        <v>3.3380909999999999</v>
       </c>
       <c r="H209" s="6">
-        <v>5.5579999999999998</v>
+        <v>4.1176120000000003</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A210" s="5" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="B210" s="6">
         <v>2022</v>
       </c>
       <c r="C210" s="6">
-        <v>55.3937983</v>
+        <v>55.453913300000004</v>
       </c>
       <c r="D210" s="6">
-        <v>-5.1951200000000002</v>
+        <v>-5.3708383</v>
       </c>
       <c r="E210" s="6">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F210" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="G210" s="6">
-        <v>5.1109999999999998</v>
+        <v>4.048</v>
       </c>
       <c r="H210" s="6">
-        <v>5.3239999999999998</v>
+        <v>4.6399999999999997</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A211" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B211" s="6">
         <v>2022</v>
       </c>
       <c r="C211" s="6">
-        <v>55.4562217</v>
+        <v>55.454524999999997</v>
       </c>
       <c r="D211" s="6">
-        <v>-5.3669700000000002</v>
+        <v>-5.3655533000000002</v>
       </c>
       <c r="E211" s="6">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F211" s="6" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="G211" s="6">
-        <v>3.3380909999999999</v>
+        <v>3.14586392</v>
       </c>
       <c r="H211" s="6">
-        <v>4.1176120000000003</v>
+        <v>3.9288204100000002</v>
       </c>
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A212" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B212" s="6">
         <v>2022</v>
       </c>
       <c r="C212" s="6">
-        <v>55.453913300000004</v>
+        <v>55.449081700000001</v>
       </c>
       <c r="D212" s="6">
-        <v>-5.3708383</v>
+        <v>-5.38985</v>
       </c>
       <c r="E212" s="6">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F212" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G212" s="6">
-        <v>4.048</v>
+        <v>4.9566299999999996</v>
       </c>
       <c r="H212" s="6">
-        <v>4.6399999999999997</v>
+        <v>5.367</v>
       </c>
     </row>
     <row r="213" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A213" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B213" s="6">
         <v>2022</v>
       </c>
       <c r="C213" s="6">
-        <v>55.454524999999997</v>
+        <v>55.448459999999997</v>
       </c>
       <c r="D213" s="6">
-        <v>-5.3655533000000002</v>
+        <v>-5.3820300000000003</v>
       </c>
       <c r="E213" s="6">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="F213" s="6" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="G213" s="6">
-        <v>3.14586392</v>
+        <v>5.4</v>
       </c>
       <c r="H213" s="6">
-        <v>3.9288204100000002</v>
+        <v>5.508534</v>
       </c>
     </row>
     <row r="214" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A214" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B214" s="6">
         <v>2022</v>
       </c>
       <c r="C214" s="6">
-        <v>55.449081700000001</v>
+        <v>55.447004999999997</v>
       </c>
       <c r="D214" s="6">
-        <v>-5.38985</v>
+        <v>-5.3888717000000002</v>
       </c>
       <c r="E214" s="6">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G214" s="6">
-        <v>4.9566299999999996</v>
+        <v>5.2220000000000004</v>
       </c>
       <c r="H214" s="6">
-        <v>5.367</v>
+        <v>5.3947149999999997</v>
       </c>
     </row>
     <row r="215" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A215" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B215" s="6">
         <v>2022</v>
       </c>
       <c r="C215" s="6">
-        <v>55.448459999999997</v>
+        <v>55.448318299999997</v>
       </c>
       <c r="D215" s="6">
-        <v>-5.3820300000000003</v>
+        <v>-5.3724083</v>
       </c>
       <c r="E215" s="6">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F215" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="G215" s="6">
-        <v>5.4</v>
+        <v>3.7554880000000002</v>
       </c>
       <c r="H215" s="6">
-        <v>5.508534</v>
+        <v>4.4162160000000004</v>
       </c>
     </row>
     <row r="216" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A216" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B216" s="6">
         <v>2022</v>
       </c>
       <c r="C216" s="6">
-        <v>55.447004999999997</v>
+        <v>55.449069999999999</v>
       </c>
       <c r="D216" s="6">
-        <v>-5.3888717000000002</v>
+        <v>-5.3661732999999998</v>
       </c>
       <c r="E216" s="6">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F216" s="6" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="G216" s="6">
-        <v>5.2220000000000004</v>
+        <v>2.668838</v>
       </c>
       <c r="H216" s="6">
-        <v>5.3947149999999997</v>
+        <v>3.5946910000000001</v>
       </c>
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A217" s="5" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B217" s="6">
         <v>2022</v>
       </c>
       <c r="C217" s="6">
-        <v>55.448318299999997</v>
+        <v>55.443755000000003</v>
       </c>
       <c r="D217" s="6">
-        <v>-5.3724083</v>
+        <v>-5.3815232999999996</v>
       </c>
       <c r="E217" s="6">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F217" s="6" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="G217" s="6">
-        <v>3.7554880000000002</v>
+        <v>3.30204999</v>
       </c>
       <c r="H217" s="6">
-        <v>4.4162160000000004</v>
+        <v>3.8502984200000001</v>
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A218" s="5" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B218" s="6">
         <v>2022</v>
       </c>
       <c r="C218" s="6">
-        <v>55.449069999999999</v>
+        <v>55.444838300000001</v>
       </c>
       <c r="D218" s="6">
-        <v>-5.3661732999999998</v>
+        <v>-5.3836550000000001</v>
       </c>
       <c r="E218" s="6">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F218" s="6" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="G218" s="6">
-        <v>2.668838</v>
+        <v>4.6828669999999999</v>
       </c>
       <c r="H218" s="6">
-        <v>3.5946910000000001</v>
+        <v>5.085693</v>
       </c>
     </row>
     <row r="219" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A219" s="5" t="s">
-        <v>189</v>
+        <v>155</v>
       </c>
       <c r="B219" s="6">
         <v>2022</v>
       </c>
       <c r="C219" s="6">
-        <v>55.443755000000003</v>
+        <v>55.442234999999997</v>
       </c>
       <c r="D219" s="6">
-        <v>-5.3815232999999996</v>
+        <v>-5.0362983000000003</v>
       </c>
       <c r="E219" s="6">
-        <v>45</v>
+        <v>125</v>
       </c>
       <c r="F219" s="6" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="G219" s="6">
-        <v>3.30204999</v>
+        <v>3.6346102999999998</v>
       </c>
       <c r="H219" s="6">
-        <v>3.8502984200000001</v>
+        <v>4.4206079699999998</v>
       </c>
     </row>
     <row r="220" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A220" s="5" t="s">
-        <v>190</v>
+        <v>156</v>
       </c>
       <c r="B220" s="6">
         <v>2022</v>
       </c>
       <c r="C220" s="6">
-        <v>55.444838300000001</v>
+        <v>55.441068299999998</v>
       </c>
       <c r="D220" s="6">
-        <v>-5.3836550000000001</v>
+        <v>-5.0364849999999999</v>
       </c>
       <c r="E220" s="6">
-        <v>51</v>
+        <v>125</v>
       </c>
       <c r="F220" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="G220" s="6">
-        <v>4.6828669999999999</v>
+        <v>3.8067813199999998</v>
       </c>
       <c r="H220" s="6">
-        <v>5.085693</v>
+        <v>4.5396766599999996</v>
       </c>
     </row>
     <row r="221" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A221" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B221" s="6">
         <v>2022</v>
       </c>
       <c r="C221" s="6">
-        <v>55.442234999999997</v>
+        <v>55.435976699999998</v>
       </c>
       <c r="D221" s="6">
-        <v>-5.0362983000000003</v>
+        <v>-5.0407549999999999</v>
       </c>
       <c r="E221" s="6">
         <v>125</v>
       </c>
       <c r="F221" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G221" s="6">
-        <v>3.6346102999999998</v>
+        <v>3.9557710500000001</v>
       </c>
       <c r="H221" s="6">
-        <v>4.4206079699999998</v>
+        <v>4.6500435700000002</v>
       </c>
     </row>
     <row r="222" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A222" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B222" s="6">
         <v>2022</v>
       </c>
       <c r="C222" s="6">
-        <v>55.441068299999998</v>
+        <v>55.436718300000003</v>
       </c>
       <c r="D222" s="6">
-        <v>-5.0364849999999999</v>
+        <v>-5.0345449999999996</v>
       </c>
       <c r="E222" s="6">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F222" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G222" s="6">
-        <v>3.8067813199999998</v>
+        <v>5.3003752799999999</v>
       </c>
       <c r="H222" s="6">
-        <v>4.5396766599999996</v>
+        <v>5.2939875699999996</v>
       </c>
     </row>
     <row r="223" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A223" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B223" s="6">
         <v>2022</v>
       </c>
       <c r="C223" s="6">
-        <v>55.435976699999998</v>
+        <v>55.434366699999998</v>
       </c>
       <c r="D223" s="6">
-        <v>-5.0407549999999999</v>
+        <v>-5.0455717</v>
       </c>
       <c r="E223" s="6">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F223" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G223" s="6">
-        <v>3.9557710500000001</v>
+        <v>3.9414613200000002</v>
       </c>
       <c r="H223" s="6">
-        <v>4.6500435700000002</v>
+        <v>4.67486581</v>
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A224" s="5" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B224" s="6">
         <v>2022</v>
       </c>
       <c r="C224" s="6">
-        <v>55.436718300000003</v>
+        <v>55.434944999999999</v>
       </c>
       <c r="D224" s="6">
-        <v>-5.0345449999999996</v>
+        <v>-5.0380916999999998</v>
       </c>
       <c r="E224" s="6">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F224" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="G224" s="6">
-        <v>5.3003752799999999</v>
+        <v>3.5526309999999999</v>
       </c>
       <c r="H224" s="6">
-        <v>5.2939875699999996</v>
+        <v>4.3330529999999996</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A225" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B225" s="6">
         <v>2022</v>
       </c>
       <c r="C225" s="6">
-        <v>55.434366699999998</v>
+        <v>55.432741700000001</v>
       </c>
       <c r="D225" s="6">
-        <v>-5.0455717</v>
+        <v>-5.0463132999999996</v>
       </c>
       <c r="E225" s="6">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F225" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G225" s="6">
-        <v>3.9414613200000002</v>
+        <v>3.9736769999999999</v>
       </c>
       <c r="H225" s="6">
-        <v>4.67486581</v>
+        <v>4.6831769999999997</v>
       </c>
     </row>
     <row r="226" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A226" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B226" s="6">
         <v>2022</v>
       </c>
       <c r="C226" s="6">
-        <v>55.434944999999999</v>
+        <v>55.431231699999998</v>
       </c>
       <c r="D226" s="6">
-        <v>-5.0380916999999998</v>
+        <v>-5.0398899999999998</v>
       </c>
       <c r="E226" s="6">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F226" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G226" s="6">
-        <v>3.5526309999999999</v>
+        <v>4.4063468300000004</v>
       </c>
       <c r="H226" s="6">
-        <v>4.3330529999999996</v>
+        <v>4.8594007599999998</v>
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A227" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B227" s="6">
         <v>2022</v>
       </c>
       <c r="C227" s="6">
-        <v>55.432741700000001</v>
+        <v>55.430316699999999</v>
       </c>
       <c r="D227" s="6">
-        <v>-5.0463132999999996</v>
+        <v>-5.0471716999999998</v>
       </c>
       <c r="E227" s="6">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F227" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G227" s="6">
-        <v>3.9736769999999999</v>
+        <v>3.9097970000000002</v>
       </c>
       <c r="H227" s="6">
-        <v>4.6831769999999997</v>
+        <v>4.5288349999999999</v>
       </c>
     </row>
     <row r="228" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A228" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B228" s="6">
         <v>2022</v>
       </c>
       <c r="C228" s="6">
-        <v>55.431231699999998</v>
+        <v>55.427759999999999</v>
       </c>
       <c r="D228" s="6">
-        <v>-5.0398899999999998</v>
+        <v>-5.0418282999999997</v>
       </c>
       <c r="E228" s="6">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F228" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G228" s="6">
-        <v>4.4063468300000004</v>
+        <v>3.9074524300000002</v>
       </c>
       <c r="H228" s="6">
-        <v>4.8594007599999998</v>
+        <v>4.6440719499999998</v>
       </c>
     </row>
     <row r="229" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A229" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="B229" s="6">
-        <v>2022</v>
-      </c>
-      <c r="C229" s="6">
-        <v>55.430316699999999</v>
-      </c>
-      <c r="D229" s="6">
-        <v>-5.0471716999999998</v>
-      </c>
-      <c r="E229" s="6">
-        <v>128</v>
-      </c>
-      <c r="F229" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="G229" s="6">
-        <v>3.9097970000000002</v>
-      </c>
-      <c r="H229" s="6">
-        <v>4.5288349999999999</v>
-      </c>
+      <c r="A229" s="2"/>
+      <c r="B229"/>
     </row>
     <row r="230" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A230" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="B230" s="6">
-        <v>2022</v>
-      </c>
-      <c r="C230" s="6">
-        <v>55.427759999999999</v>
-      </c>
-      <c r="D230" s="6">
-        <v>-5.0418282999999997</v>
-      </c>
-      <c r="E230" s="6">
-        <v>123</v>
-      </c>
-      <c r="F230" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="G230" s="6">
-        <v>3.9074524300000002</v>
-      </c>
-      <c r="H230" s="6">
-        <v>4.6440719499999998</v>
-      </c>
+      <c r="A230" s="2"/>
+      <c r="B230"/>
     </row>
     <row r="231" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A231" s="2"/>
       <c r="B231"/>
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A232" s="2"/>
       <c r="B232"/>
     </row>
     <row r="233" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A233" s="2"/>
       <c r="B233"/>
     </row>
     <row r="234" spans="1:8" x14ac:dyDescent="0.2">
@@ -7187,12 +7117,6 @@
     </row>
     <row r="236" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B236"/>
-    </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B237"/>
-    </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B238"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>